<commit_message>
Add nap count evolution chart; sample goes from 5 to 3 naps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vb4xjN4NNLsKRyCx58QePR
</commit_message>
<xml_diff>
--- a/static/sample-sleep-log.xlsx
+++ b/static/sample-sleep-log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E119"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -428,10 +428,10 @@
         <v>2026-09-01</v>
       </c>
       <c r="B2" t="str">
-        <v>08:40</v>
+        <v>08:15</v>
       </c>
       <c r="C2" t="str">
-        <v>09:46</v>
+        <v>09:03</v>
       </c>
       <c r="D2" t="str">
         <v>Nap</v>
@@ -445,10 +445,10 @@
         <v>2026-09-01</v>
       </c>
       <c r="B3" t="str">
-        <v>11:52</v>
+        <v>10:39</v>
       </c>
       <c r="C3" t="str">
-        <v>12:23</v>
+        <v>11:05</v>
       </c>
       <c r="D3" t="str">
         <v>Nap</v>
@@ -462,10 +462,10 @@
         <v>2026-09-01</v>
       </c>
       <c r="B4" t="str">
-        <v>15:09</v>
+        <v>13:07</v>
       </c>
       <c r="C4" t="str">
-        <v>15:56</v>
+        <v>13:43</v>
       </c>
       <c r="D4" t="str">
         <v>Nap</v>
@@ -479,10 +479,10 @@
         <v>2026-09-01</v>
       </c>
       <c r="B5" t="str">
-        <v>17:08</v>
+        <v>14:55</v>
       </c>
       <c r="C5" t="str">
-        <v>18:06</v>
+        <v>15:38</v>
       </c>
       <c r="D5" t="str">
         <v>Nap</v>
@@ -496,16 +496,16 @@
         <v>2026-09-01</v>
       </c>
       <c r="B6" t="str">
-        <v>19:43</v>
+        <v>17:08</v>
       </c>
       <c r="C6" t="str">
-        <v>01:43</v>
+        <v>17:44</v>
       </c>
       <c r="D6" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E6" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -513,30 +513,30 @@
         <v>2026-09-01</v>
       </c>
       <c r="B7" t="str">
-        <v>01:53</v>
+        <v>19:39</v>
       </c>
       <c r="C7" t="str">
-        <v>06:53</v>
+        <v>00:55</v>
       </c>
       <c r="D7" t="str">
         <v>Night</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-09-02</v>
+        <v>2026-09-01</v>
       </c>
       <c r="B8" t="str">
-        <v>08:55</v>
+        <v>01:14</v>
       </c>
       <c r="C8" t="str">
-        <v>09:50</v>
+        <v>06:30</v>
       </c>
       <c r="D8" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -547,10 +547,10 @@
         <v>2026-09-02</v>
       </c>
       <c r="B9" t="str">
-        <v>12:08</v>
+        <v>08:36</v>
       </c>
       <c r="C9" t="str">
-        <v>12:31</v>
+        <v>08:58</v>
       </c>
       <c r="D9" t="str">
         <v>Nap</v>
@@ -564,10 +564,10 @@
         <v>2026-09-02</v>
       </c>
       <c r="B10" t="str">
-        <v>15:07</v>
+        <v>10:51</v>
       </c>
       <c r="C10" t="str">
-        <v>15:50</v>
+        <v>11:25</v>
       </c>
       <c r="D10" t="str">
         <v>Nap</v>
@@ -581,10 +581,10 @@
         <v>2026-09-02</v>
       </c>
       <c r="B11" t="str">
-        <v>17:32</v>
+        <v>13:13</v>
       </c>
       <c r="C11" t="str">
-        <v>18:32</v>
+        <v>13:57</v>
       </c>
       <c r="D11" t="str">
         <v>Nap</v>
@@ -598,16 +598,16 @@
         <v>2026-09-02</v>
       </c>
       <c r="B12" t="str">
-        <v>19:11</v>
+        <v>14:49</v>
       </c>
       <c r="C12" t="str">
-        <v>01:16</v>
+        <v>15:24</v>
       </c>
       <c r="D12" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E12" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -615,13 +615,13 @@
         <v>2026-09-02</v>
       </c>
       <c r="B13" t="str">
-        <v>01:33</v>
+        <v>17:13</v>
       </c>
       <c r="C13" t="str">
-        <v>06:56</v>
+        <v>17:54</v>
       </c>
       <c r="D13" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -629,33 +629,33 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-09-03</v>
+        <v>2026-09-02</v>
       </c>
       <c r="B14" t="str">
-        <v>09:16</v>
+        <v>19:37</v>
       </c>
       <c r="C14" t="str">
-        <v>10:21</v>
+        <v>01:14</v>
       </c>
       <c r="D14" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-09-03</v>
+        <v>2026-09-02</v>
       </c>
       <c r="B15" t="str">
-        <v>11:55</v>
+        <v>01:26</v>
       </c>
       <c r="C15" t="str">
-        <v>12:32</v>
+        <v>07:10</v>
       </c>
       <c r="D15" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -666,10 +666,10 @@
         <v>2026-09-03</v>
       </c>
       <c r="B16" t="str">
-        <v>15:13</v>
+        <v>08:40</v>
       </c>
       <c r="C16" t="str">
-        <v>15:50</v>
+        <v>09:10</v>
       </c>
       <c r="D16" t="str">
         <v>Nap</v>
@@ -683,10 +683,10 @@
         <v>2026-09-03</v>
       </c>
       <c r="B17" t="str">
-        <v>17:01</v>
+        <v>10:35</v>
       </c>
       <c r="C17" t="str">
-        <v>17:36</v>
+        <v>11:04</v>
       </c>
       <c r="D17" t="str">
         <v>Nap</v>
@@ -700,16 +700,16 @@
         <v>2026-09-03</v>
       </c>
       <c r="B18" t="str">
-        <v>19:26</v>
+        <v>12:58</v>
       </c>
       <c r="C18" t="str">
-        <v>01:25</v>
+        <v>13:27</v>
       </c>
       <c r="D18" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E18" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -717,13 +717,13 @@
         <v>2026-09-03</v>
       </c>
       <c r="B19" t="str">
-        <v>01:48</v>
+        <v>15:13</v>
       </c>
       <c r="C19" t="str">
-        <v>06:48</v>
+        <v>15:50</v>
       </c>
       <c r="D19" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -731,13 +731,13 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-03</v>
       </c>
       <c r="B20" t="str">
-        <v>08:42</v>
+        <v>17:07</v>
       </c>
       <c r="C20" t="str">
-        <v>09:16</v>
+        <v>17:53</v>
       </c>
       <c r="D20" t="str">
         <v>Nap</v>
@@ -748,33 +748,33 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-03</v>
       </c>
       <c r="B21" t="str">
-        <v>12:02</v>
+        <v>19:08</v>
       </c>
       <c r="C21" t="str">
-        <v>12:47</v>
+        <v>00:51</v>
       </c>
       <c r="D21" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E21" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-03</v>
       </c>
       <c r="B22" t="str">
-        <v>14:57</v>
+        <v>01:00</v>
       </c>
       <c r="C22" t="str">
-        <v>15:27</v>
+        <v>06:46</v>
       </c>
       <c r="D22" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -785,10 +785,10 @@
         <v>2026-09-04</v>
       </c>
       <c r="B23" t="str">
-        <v>17:31</v>
+        <v>08:42</v>
       </c>
       <c r="C23" t="str">
-        <v>17:54</v>
+        <v>09:04</v>
       </c>
       <c r="D23" t="str">
         <v>Nap</v>
@@ -802,16 +802,16 @@
         <v>2026-09-04</v>
       </c>
       <c r="B24" t="str">
-        <v>19:23</v>
+        <v>10:41</v>
       </c>
       <c r="C24" t="str">
-        <v>01:18</v>
+        <v>11:11</v>
       </c>
       <c r="D24" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E24" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -819,13 +819,13 @@
         <v>2026-09-04</v>
       </c>
       <c r="B25" t="str">
-        <v>01:26</v>
+        <v>13:05</v>
       </c>
       <c r="C25" t="str">
-        <v>07:10</v>
+        <v>13:53</v>
       </c>
       <c r="D25" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -833,13 +833,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B26" t="str">
-        <v>08:56</v>
+        <v>15:00</v>
       </c>
       <c r="C26" t="str">
-        <v>09:30</v>
+        <v>15:25</v>
       </c>
       <c r="D26" t="str">
         <v>Nap</v>
@@ -850,13 +850,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B27" t="str">
-        <v>11:55</v>
+        <v>16:57</v>
       </c>
       <c r="C27" t="str">
-        <v>12:36</v>
+        <v>17:26</v>
       </c>
       <c r="D27" t="str">
         <v>Nap</v>
@@ -867,33 +867,33 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B28" t="str">
-        <v>14:53</v>
+        <v>19:23</v>
       </c>
       <c r="C28" t="str">
-        <v>15:40</v>
+        <v>23:20</v>
       </c>
       <c r="D28" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E28" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B29" t="str">
-        <v>17:20</v>
+        <v>23:30</v>
       </c>
       <c r="C29" t="str">
-        <v>17:52</v>
+        <v>03:51</v>
       </c>
       <c r="D29" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -901,19 +901,19 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B30" t="str">
-        <v>19:50</v>
+        <v>04:05</v>
       </c>
       <c r="C30" t="str">
-        <v>01:33</v>
+        <v>06:47</v>
       </c>
       <c r="D30" t="str">
         <v>Night</v>
       </c>
       <c r="E30" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -921,13 +921,13 @@
         <v>2026-09-05</v>
       </c>
       <c r="B31" t="str">
-        <v>01:48</v>
+        <v>09:11</v>
       </c>
       <c r="C31" t="str">
-        <v>06:53</v>
+        <v>10:05</v>
       </c>
       <c r="D31" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -935,13 +935,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B32" t="str">
-        <v>09:00</v>
+        <v>12:04</v>
       </c>
       <c r="C32" t="str">
-        <v>09:54</v>
+        <v>12:54</v>
       </c>
       <c r="D32" t="str">
         <v>Nap</v>
@@ -952,13 +952,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B33" t="str">
-        <v>12:18</v>
+        <v>15:00</v>
       </c>
       <c r="C33" t="str">
-        <v>12:58</v>
+        <v>15:56</v>
       </c>
       <c r="D33" t="str">
         <v>Nap</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B34" t="str">
-        <v>15:08</v>
+        <v>17:28</v>
       </c>
       <c r="C34" t="str">
-        <v>15:41</v>
+        <v>18:15</v>
       </c>
       <c r="D34" t="str">
         <v>Nap</v>
@@ -986,36 +986,36 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B35" t="str">
-        <v>17:18</v>
+        <v>19:40</v>
       </c>
       <c r="C35" t="str">
-        <v>17:56</v>
+        <v>00:54</v>
       </c>
       <c r="D35" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E35" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B36" t="str">
-        <v>19:22</v>
+        <v>01:07</v>
       </c>
       <c r="C36" t="str">
-        <v>00:44</v>
+        <v>06:36</v>
       </c>
       <c r="D36" t="str">
         <v>Night</v>
       </c>
       <c r="E36" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -1023,13 +1023,13 @@
         <v>2026-09-06</v>
       </c>
       <c r="B37" t="str">
-        <v>01:05</v>
+        <v>08:39</v>
       </c>
       <c r="C37" t="str">
-        <v>07:08</v>
+        <v>09:25</v>
       </c>
       <c r="D37" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -1037,13 +1037,13 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B38" t="str">
-        <v>08:43</v>
+        <v>10:33</v>
       </c>
       <c r="C38" t="str">
-        <v>09:23</v>
+        <v>11:18</v>
       </c>
       <c r="D38" t="str">
         <v>Nap</v>
@@ -1054,13 +1054,13 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B39" t="str">
-        <v>11:46</v>
+        <v>12:47</v>
       </c>
       <c r="C39" t="str">
-        <v>12:10</v>
+        <v>13:19</v>
       </c>
       <c r="D39" t="str">
         <v>Nap</v>
@@ -1071,13 +1071,13 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B40" t="str">
-        <v>15:20</v>
+        <v>14:50</v>
       </c>
       <c r="C40" t="str">
-        <v>15:51</v>
+        <v>15:12</v>
       </c>
       <c r="D40" t="str">
         <v>Nap</v>
@@ -1088,13 +1088,13 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B41" t="str">
-        <v>17:20</v>
+        <v>17:15</v>
       </c>
       <c r="C41" t="str">
-        <v>17:47</v>
+        <v>17:42</v>
       </c>
       <c r="D41" t="str">
         <v>Nap</v>
@@ -1105,33 +1105,33 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B42" t="str">
-        <v>19:28</v>
+        <v>19:37</v>
       </c>
       <c r="C42" t="str">
-        <v>06:23</v>
+        <v>00:45</v>
       </c>
       <c r="D42" t="str">
         <v>Night</v>
       </c>
       <c r="E42" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B43" t="str">
-        <v>09:17</v>
+        <v>01:08</v>
       </c>
       <c r="C43" t="str">
-        <v>10:21</v>
+        <v>06:51</v>
       </c>
       <c r="D43" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E43" t="str">
         <v/>
@@ -1139,13 +1139,13 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B44" t="str">
-        <v>12:16</v>
+        <v>09:12</v>
       </c>
       <c r="C44" t="str">
-        <v>13:20</v>
+        <v>10:14</v>
       </c>
       <c r="D44" t="str">
         <v>Nap</v>
@@ -1156,13 +1156,13 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B45" t="str">
-        <v>15:16</v>
+        <v>12:12</v>
       </c>
       <c r="C45" t="str">
-        <v>16:14</v>
+        <v>13:14</v>
       </c>
       <c r="D45" t="str">
         <v>Nap</v>
@@ -1173,13 +1173,13 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B46" t="str">
-        <v>17:06</v>
+        <v>15:08</v>
       </c>
       <c r="C46" t="str">
-        <v>17:27</v>
+        <v>15:51</v>
       </c>
       <c r="D46" t="str">
         <v>Nap</v>
@@ -1190,47 +1190,47 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B47" t="str">
-        <v>19:17</v>
+        <v>17:00</v>
       </c>
       <c r="C47" t="str">
-        <v>22:48</v>
+        <v>17:42</v>
       </c>
       <c r="D47" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E47" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B48" t="str">
-        <v>23:08</v>
+        <v>19:09</v>
       </c>
       <c r="C48" t="str">
-        <v>02:58</v>
+        <v>01:08</v>
       </c>
       <c r="D48" t="str">
         <v>Night</v>
       </c>
       <c r="E48" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B49" t="str">
-        <v>03:17</v>
+        <v>01:23</v>
       </c>
       <c r="C49" t="str">
-        <v>06:52</v>
+        <v>06:29</v>
       </c>
       <c r="D49" t="str">
         <v>Night</v>
@@ -1241,13 +1241,13 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-08</v>
       </c>
       <c r="B50" t="str">
-        <v>08:50</v>
+        <v>09:06</v>
       </c>
       <c r="C50" t="str">
-        <v>09:54</v>
+        <v>09:48</v>
       </c>
       <c r="D50" t="str">
         <v>Nap</v>
@@ -1258,13 +1258,13 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-08</v>
       </c>
       <c r="B51" t="str">
-        <v>11:49</v>
+        <v>12:11</v>
       </c>
       <c r="C51" t="str">
-        <v>12:28</v>
+        <v>12:53</v>
       </c>
       <c r="D51" t="str">
         <v>Nap</v>
@@ -1275,13 +1275,13 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-08</v>
       </c>
       <c r="B52" t="str">
-        <v>15:16</v>
+        <v>14:56</v>
       </c>
       <c r="C52" t="str">
-        <v>15:42</v>
+        <v>15:58</v>
       </c>
       <c r="D52" t="str">
         <v>Nap</v>
@@ -1292,13 +1292,13 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-08</v>
       </c>
       <c r="B53" t="str">
-        <v>17:15</v>
+        <v>17:04</v>
       </c>
       <c r="C53" t="str">
-        <v>17:35</v>
+        <v>17:54</v>
       </c>
       <c r="D53" t="str">
         <v>Nap</v>
@@ -1309,13 +1309,13 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-08</v>
       </c>
       <c r="B54" t="str">
-        <v>19:51</v>
+        <v>19:05</v>
       </c>
       <c r="C54" t="str">
-        <v>07:10</v>
+        <v>06:53</v>
       </c>
       <c r="D54" t="str">
         <v>Night</v>
@@ -1326,13 +1326,13 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B55" t="str">
-        <v>08:41</v>
+        <v>09:13</v>
       </c>
       <c r="C55" t="str">
-        <v>09:46</v>
+        <v>09:49</v>
       </c>
       <c r="D55" t="str">
         <v>Nap</v>
@@ -1343,13 +1343,13 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B56" t="str">
-        <v>11:48</v>
+        <v>12:12</v>
       </c>
       <c r="C56" t="str">
-        <v>12:56</v>
+        <v>12:53</v>
       </c>
       <c r="D56" t="str">
         <v>Nap</v>
@@ -1360,13 +1360,13 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B57" t="str">
-        <v>15:03</v>
+        <v>15:14</v>
       </c>
       <c r="C57" t="str">
-        <v>15:57</v>
+        <v>16:06</v>
       </c>
       <c r="D57" t="str">
         <v>Nap</v>
@@ -1377,13 +1377,13 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B58" t="str">
-        <v>17:06</v>
+        <v>17:20</v>
       </c>
       <c r="C58" t="str">
-        <v>17:37</v>
+        <v>18:03</v>
       </c>
       <c r="D58" t="str">
         <v>Nap</v>
@@ -1394,33 +1394,33 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B59" t="str">
-        <v>19:15</v>
+        <v>19:16</v>
       </c>
       <c r="C59" t="str">
-        <v>06:18</v>
+        <v>01:09</v>
       </c>
       <c r="D59" t="str">
         <v>Night</v>
       </c>
       <c r="E59" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B60" t="str">
-        <v>09:26</v>
+        <v>01:28</v>
       </c>
       <c r="C60" t="str">
-        <v>10:46</v>
+        <v>06:18</v>
       </c>
       <c r="D60" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -1428,13 +1428,13 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-10</v>
       </c>
       <c r="B61" t="str">
-        <v>13:09</v>
+        <v>09:06</v>
       </c>
       <c r="C61" t="str">
-        <v>14:19</v>
+        <v>09:56</v>
       </c>
       <c r="D61" t="str">
         <v>Nap</v>
@@ -1445,13 +1445,13 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-10</v>
       </c>
       <c r="B62" t="str">
-        <v>15:56</v>
+        <v>11:46</v>
       </c>
       <c r="C62" t="str">
-        <v>16:47</v>
+        <v>12:24</v>
       </c>
       <c r="D62" t="str">
         <v>Nap</v>
@@ -1462,33 +1462,33 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-10</v>
       </c>
       <c r="B63" t="str">
-        <v>19:51</v>
+        <v>15:13</v>
       </c>
       <c r="C63" t="str">
-        <v>00:53</v>
+        <v>15:52</v>
       </c>
       <c r="D63" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E63" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-10</v>
       </c>
       <c r="B64" t="str">
-        <v>01:16</v>
+        <v>17:21</v>
       </c>
       <c r="C64" t="str">
-        <v>07:09</v>
+        <v>18:23</v>
       </c>
       <c r="D64" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E64" t="str">
         <v/>
@@ -1496,16 +1496,16 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-09-12</v>
+        <v>2026-09-10</v>
       </c>
       <c r="B65" t="str">
-        <v>09:29</v>
+        <v>19:07</v>
       </c>
       <c r="C65" t="str">
-        <v>11:04</v>
+        <v>07:07</v>
       </c>
       <c r="D65" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E65" t="str">
         <v/>
@@ -1513,13 +1513,13 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-09-12</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B66" t="str">
-        <v>13:18</v>
+        <v>09:30</v>
       </c>
       <c r="C66" t="str">
-        <v>14:41</v>
+        <v>10:54</v>
       </c>
       <c r="D66" t="str">
         <v>Nap</v>
@@ -1530,13 +1530,13 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-09-12</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B67" t="str">
-        <v>16:12</v>
+        <v>13:08</v>
       </c>
       <c r="C67" t="str">
-        <v>17:09</v>
+        <v>14:16</v>
       </c>
       <c r="D67" t="str">
         <v>Nap</v>
@@ -1547,16 +1547,16 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-09-12</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B68" t="str">
-        <v>19:41</v>
+        <v>16:07</v>
       </c>
       <c r="C68" t="str">
-        <v>06:39</v>
+        <v>17:24</v>
       </c>
       <c r="D68" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E68" t="str">
         <v/>
@@ -1564,33 +1564,33 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-09-13</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B69" t="str">
-        <v>09:04</v>
+        <v>19:49</v>
       </c>
       <c r="C69" t="str">
-        <v>10:09</v>
+        <v>23:57</v>
       </c>
       <c r="D69" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E69" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-09-13</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B70" t="str">
-        <v>13:15</v>
+        <v>00:13</v>
       </c>
       <c r="C70" t="str">
-        <v>14:28</v>
+        <v>03:37</v>
       </c>
       <c r="D70" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E70" t="str">
         <v/>
@@ -1598,16 +1598,16 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-09-13</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B71" t="str">
-        <v>16:09</v>
+        <v>03:54</v>
       </c>
       <c r="C71" t="str">
-        <v>17:25</v>
+        <v>06:39</v>
       </c>
       <c r="D71" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E71" t="str">
         <v/>
@@ -1615,33 +1615,33 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-09-13</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B72" t="str">
-        <v>19:42</v>
+        <v>09:07</v>
       </c>
       <c r="C72" t="str">
-        <v>00:47</v>
+        <v>09:52</v>
       </c>
       <c r="D72" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E72" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-09-13</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B73" t="str">
-        <v>00:58</v>
+        <v>12:07</v>
       </c>
       <c r="C73" t="str">
-        <v>06:40</v>
+        <v>12:55</v>
       </c>
       <c r="D73" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E73" t="str">
         <v/>
@@ -1649,13 +1649,13 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B74" t="str">
-        <v>09:34</v>
+        <v>14:51</v>
       </c>
       <c r="C74" t="str">
-        <v>11:09</v>
+        <v>15:35</v>
       </c>
       <c r="D74" t="str">
         <v>Nap</v>
@@ -1666,13 +1666,13 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B75" t="str">
-        <v>13:05</v>
+        <v>17:30</v>
       </c>
       <c r="C75" t="str">
-        <v>14:34</v>
+        <v>18:35</v>
       </c>
       <c r="D75" t="str">
         <v>Nap</v>
@@ -1683,16 +1683,16 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B76" t="str">
-        <v>16:32</v>
+        <v>19:37</v>
       </c>
       <c r="C76" t="str">
-        <v>17:27</v>
+        <v>07:10</v>
       </c>
       <c r="D76" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E76" t="str">
         <v/>
@@ -1700,33 +1700,33 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-13</v>
       </c>
       <c r="B77" t="str">
-        <v>19:37</v>
+        <v>08:51</v>
       </c>
       <c r="C77" t="str">
-        <v>01:35</v>
+        <v>09:45</v>
       </c>
       <c r="D77" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E77" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-13</v>
       </c>
       <c r="B78" t="str">
-        <v>01:59</v>
+        <v>11:49</v>
       </c>
       <c r="C78" t="str">
-        <v>06:48</v>
+        <v>12:39</v>
       </c>
       <c r="D78" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E78" t="str">
         <v/>
@@ -1734,13 +1734,13 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-13</v>
       </c>
       <c r="B79" t="str">
-        <v>09:14</v>
+        <v>15:02</v>
       </c>
       <c r="C79" t="str">
-        <v>10:08</v>
+        <v>16:00</v>
       </c>
       <c r="D79" t="str">
         <v>Nap</v>
@@ -1751,13 +1751,13 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-13</v>
       </c>
       <c r="B80" t="str">
-        <v>12:58</v>
+        <v>17:28</v>
       </c>
       <c r="C80" t="str">
-        <v>13:51</v>
+        <v>18:17</v>
       </c>
       <c r="D80" t="str">
         <v>Nap</v>
@@ -1768,16 +1768,16 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-13</v>
       </c>
       <c r="B81" t="str">
-        <v>16:22</v>
+        <v>19:14</v>
       </c>
       <c r="C81" t="str">
-        <v>17:33</v>
+        <v>06:25</v>
       </c>
       <c r="D81" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E81" t="str">
         <v/>
@@ -1785,16 +1785,16 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-14</v>
       </c>
       <c r="B82" t="str">
-        <v>19:33</v>
+        <v>09:20</v>
       </c>
       <c r="C82" t="str">
-        <v>07:00</v>
+        <v>10:31</v>
       </c>
       <c r="D82" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E82" t="str">
         <v/>
@@ -1802,13 +1802,13 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-14</v>
       </c>
       <c r="B83" t="str">
-        <v>09:09</v>
+        <v>13:02</v>
       </c>
       <c r="C83" t="str">
-        <v>10:32</v>
+        <v>14:12</v>
       </c>
       <c r="D83" t="str">
         <v>Nap</v>
@@ -1819,13 +1819,13 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-14</v>
       </c>
       <c r="B84" t="str">
-        <v>12:41</v>
+        <v>16:23</v>
       </c>
       <c r="C84" t="str">
-        <v>13:41</v>
+        <v>17:29</v>
       </c>
       <c r="D84" t="str">
         <v>Nap</v>
@@ -1836,47 +1836,47 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-14</v>
       </c>
       <c r="B85" t="str">
-        <v>16:17</v>
+        <v>19:43</v>
       </c>
       <c r="C85" t="str">
-        <v>17:12</v>
+        <v>23:01</v>
       </c>
       <c r="D85" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E85" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-14</v>
       </c>
       <c r="B86" t="str">
-        <v>19:41</v>
+        <v>23:20</v>
       </c>
       <c r="C86" t="str">
-        <v>23:20</v>
+        <v>02:44</v>
       </c>
       <c r="D86" t="str">
         <v>Night</v>
       </c>
       <c r="E86" t="str">
-        <v>Feed</v>
+        <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-14</v>
       </c>
       <c r="B87" t="str">
-        <v>23:27</v>
+        <v>02:54</v>
       </c>
       <c r="C87" t="str">
-        <v>03:33</v>
+        <v>06:48</v>
       </c>
       <c r="D87" t="str">
         <v>Night</v>
@@ -1887,16 +1887,16 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-15</v>
       </c>
       <c r="B88" t="str">
-        <v>03:54</v>
+        <v>09:20</v>
       </c>
       <c r="C88" t="str">
-        <v>06:55</v>
+        <v>10:28</v>
       </c>
       <c r="D88" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E88" t="str">
         <v/>
@@ -1904,13 +1904,13 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-15</v>
       </c>
       <c r="B89" t="str">
-        <v>09:32</v>
+        <v>12:47</v>
       </c>
       <c r="C89" t="str">
-        <v>11:03</v>
+        <v>14:05</v>
       </c>
       <c r="D89" t="str">
         <v>Nap</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-15</v>
       </c>
       <c r="B90" t="str">
-        <v>13:07</v>
+        <v>16:25</v>
       </c>
       <c r="C90" t="str">
-        <v>14:40</v>
+        <v>17:47</v>
       </c>
       <c r="D90" t="str">
         <v>Nap</v>
@@ -1938,16 +1938,16 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-15</v>
       </c>
       <c r="B91" t="str">
-        <v>15:56</v>
+        <v>19:51</v>
       </c>
       <c r="C91" t="str">
-        <v>17:19</v>
+        <v>07:13</v>
       </c>
       <c r="D91" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E91" t="str">
         <v/>
@@ -1955,16 +1955,16 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2026-09-17</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B92" t="str">
-        <v>19:35</v>
+        <v>09:01</v>
       </c>
       <c r="C92" t="str">
-        <v>07:09</v>
+        <v>10:19</v>
       </c>
       <c r="D92" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E92" t="str">
         <v/>
@@ -1972,13 +1972,13 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>2026-09-18</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B93" t="str">
-        <v>08:56</v>
+        <v>13:03</v>
       </c>
       <c r="C93" t="str">
-        <v>09:48</v>
+        <v>14:20</v>
       </c>
       <c r="D93" t="str">
         <v>Nap</v>
@@ -1989,13 +1989,13 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>2026-09-18</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B94" t="str">
-        <v>12:43</v>
+        <v>16:27</v>
       </c>
       <c r="C94" t="str">
-        <v>13:33</v>
+        <v>17:23</v>
       </c>
       <c r="D94" t="str">
         <v>Nap</v>
@@ -2006,30 +2006,30 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>2026-09-18</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B95" t="str">
-        <v>15:58</v>
+        <v>19:12</v>
       </c>
       <c r="C95" t="str">
-        <v>16:43</v>
+        <v>22:16</v>
       </c>
       <c r="D95" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E95" t="str">
-        <v/>
+        <v>Feed</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>2026-09-18</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B96" t="str">
-        <v>19:35</v>
+        <v>22:33</v>
       </c>
       <c r="C96" t="str">
-        <v>06:27</v>
+        <v>02:51</v>
       </c>
       <c r="D96" t="str">
         <v>Night</v>
@@ -2040,16 +2040,16 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B97" t="str">
-        <v>09:00</v>
+        <v>03:00</v>
       </c>
       <c r="C97" t="str">
-        <v>09:55</v>
+        <v>06:20</v>
       </c>
       <c r="D97" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E97" t="str">
         <v/>
@@ -2057,13 +2057,13 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B98" t="str">
-        <v>13:07</v>
+        <v>09:04</v>
       </c>
       <c r="C98" t="str">
-        <v>14:04</v>
+        <v>10:05</v>
       </c>
       <c r="D98" t="str">
         <v>Nap</v>
@@ -2074,13 +2074,13 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B99" t="str">
-        <v>16:13</v>
+        <v>13:05</v>
       </c>
       <c r="C99" t="str">
-        <v>17:48</v>
+        <v>14:07</v>
       </c>
       <c r="D99" t="str">
         <v>Nap</v>
@@ -2091,16 +2091,16 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B100" t="str">
-        <v>19:26</v>
+        <v>16:14</v>
       </c>
       <c r="C100" t="str">
-        <v>07:01</v>
+        <v>17:39</v>
       </c>
       <c r="D100" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E100" t="str">
         <v/>
@@ -2108,16 +2108,16 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B101" t="str">
-        <v>09:11</v>
+        <v>19:26</v>
       </c>
       <c r="C101" t="str">
-        <v>10:17</v>
+        <v>07:01</v>
       </c>
       <c r="D101" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E101" t="str">
         <v/>
@@ -2125,13 +2125,13 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-18</v>
       </c>
       <c r="B102" t="str">
-        <v>12:42</v>
+        <v>09:12</v>
       </c>
       <c r="C102" t="str">
-        <v>13:39</v>
+        <v>10:19</v>
       </c>
       <c r="D102" t="str">
         <v>Nap</v>
@@ -2142,13 +2142,13 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-18</v>
       </c>
       <c r="B103" t="str">
-        <v>16:27</v>
+        <v>12:47</v>
       </c>
       <c r="C103" t="str">
-        <v>18:01</v>
+        <v>13:49</v>
       </c>
       <c r="D103" t="str">
         <v>Nap</v>
@@ -2159,16 +2159,16 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-18</v>
       </c>
       <c r="B104" t="str">
-        <v>19:13</v>
+        <v>16:24</v>
       </c>
       <c r="C104" t="str">
-        <v>06:46</v>
+        <v>17:48</v>
       </c>
       <c r="D104" t="str">
-        <v>Night</v>
+        <v>Nap</v>
       </c>
       <c r="E104" t="str">
         <v/>
@@ -2176,16 +2176,16 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>2026-09-21</v>
+        <v>2026-09-18</v>
       </c>
       <c r="B105" t="str">
-        <v>09:00</v>
+        <v>19:13</v>
       </c>
       <c r="C105" t="str">
-        <v>09:56</v>
+        <v>06:46</v>
       </c>
       <c r="D105" t="str">
-        <v>Nap</v>
+        <v>Night</v>
       </c>
       <c r="E105" t="str">
         <v/>
@@ -2193,13 +2193,13 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>2026-09-21</v>
+        <v>2026-09-19</v>
       </c>
       <c r="B106" t="str">
-        <v>13:04</v>
+        <v>09:04</v>
       </c>
       <c r="C106" t="str">
-        <v>13:58</v>
+        <v>10:05</v>
       </c>
       <c r="D106" t="str">
         <v>Nap</v>
@@ -2210,13 +2210,13 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>2026-09-21</v>
+        <v>2026-09-19</v>
       </c>
       <c r="B107" t="str">
-        <v>15:58</v>
+        <v>13:03</v>
       </c>
       <c r="C107" t="str">
-        <v>16:57</v>
+        <v>14:03</v>
       </c>
       <c r="D107" t="str">
         <v>Nap</v>
@@ -2227,24 +2227,211 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B108" t="str">
+        <v>16:02</v>
+      </c>
+      <c r="C108" t="str">
+        <v>17:05</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="E108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B109" t="str">
+        <v>19:37</v>
+      </c>
+      <c r="C109" t="str">
+        <v>06:44</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Night</v>
+      </c>
+      <c r="E109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B110" t="str">
+        <v>09:30</v>
+      </c>
+      <c r="C110" t="str">
+        <v>10:27</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="E110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B111" t="str">
+        <v>12:57</v>
+      </c>
+      <c r="C111" t="str">
+        <v>14:01</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="E111" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B112" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C112" t="str">
+        <v>16:55</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="E112" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B113" t="str">
+        <v>19:26</v>
+      </c>
+      <c r="C113" t="str">
+        <v>23:43</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Night</v>
+      </c>
+      <c r="E113" t="str">
+        <v>Feed</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B114" t="str">
+        <v>00:03</v>
+      </c>
+      <c r="C114" t="str">
+        <v>03:52</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Night</v>
+      </c>
+      <c r="E114" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B115" t="str">
+        <v>04:14</v>
+      </c>
+      <c r="C115" t="str">
+        <v>07:10</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Night</v>
+      </c>
+      <c r="E115" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
         <v>2026-09-21</v>
       </c>
-      <c r="B108" t="str">
-        <v>19:37</v>
-      </c>
-      <c r="C108" t="str">
-        <v>06:44</v>
-      </c>
-      <c r="D108" t="str">
-        <v>Night</v>
-      </c>
-      <c r="E108" t="str">
+      <c r="B116" t="str">
+        <v>09:29</v>
+      </c>
+      <c r="C116" t="str">
+        <v>10:48</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="E116" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B117" t="str">
+        <v>13:05</v>
+      </c>
+      <c r="C117" t="str">
+        <v>14:17</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="E117" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B118" t="str">
+        <v>16:10</v>
+      </c>
+      <c r="C118" t="str">
+        <v>17:17</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="E118" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B119" t="str">
+        <v>19:30</v>
+      </c>
+      <c r="C119" t="str">
+        <v>06:49</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Night</v>
+      </c>
+      <c r="E119" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E108"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E119"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Switch charts to Plotly, add sleep entry form, newest-first timeline
- Interactive Plotly charts (zoom, unified hover, smooth lines, range
  buttons) themed from the CSS color tokens, lazy-loaded
- Form to add sleeps on the site, saved in the browser, combined with
  uploaded data, exportable to Excel and readable again
- Simple layout accepts settling start, method and mood columns; sample
  data includes them
- Lines and areas break across missing days and weeks
- Timeline lists days newest first with today on top

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vb4xjN4NNLsKRyCx58QePR
</commit_message>
<xml_diff>
--- a/static/sample-sleep-log.xlsx
+++ b/static/sample-sleep-log.xlsx
@@ -397,13 +397,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E119"/>
+  <dimension ref="A1:H117"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" customWidth="1"/>
+    <col min="5" max="5" width="7.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -411,15 +414,24 @@
         <v>Date</v>
       </c>
       <c r="B1" t="str">
-        <v>Start</v>
+        <v>Settling start</v>
       </c>
       <c r="C1" t="str">
-        <v>End</v>
+        <v>Fell asleep</v>
       </c>
       <c r="D1" t="str">
+        <v>Woke up</v>
+      </c>
+      <c r="E1" t="str">
         <v>Type</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
+        <v>How fell asleep</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Mood after</v>
+      </c>
+      <c r="H1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -428,15 +440,24 @@
         <v>2026-09-01</v>
       </c>
       <c r="B2" t="str">
+        <v>07:57</v>
+      </c>
+      <c r="C2" t="str">
         <v>08:15</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>09:03</v>
       </c>
-      <c r="D2" t="str">
-        <v>Nap</v>
-      </c>
       <c r="E2" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H2" t="str">
         <v/>
       </c>
     </row>
@@ -445,15 +466,24 @@
         <v>2026-09-01</v>
       </c>
       <c r="B3" t="str">
-        <v>10:39</v>
+        <v>10:23</v>
       </c>
       <c r="C3" t="str">
-        <v>11:05</v>
+        <v>10:46</v>
       </c>
       <c r="D3" t="str">
-        <v>Nap</v>
+        <v>11:16</v>
       </c>
       <c r="E3" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H3" t="str">
         <v/>
       </c>
     </row>
@@ -462,15 +492,24 @@
         <v>2026-09-01</v>
       </c>
       <c r="B4" t="str">
-        <v>13:07</v>
+        <v>12:43</v>
       </c>
       <c r="C4" t="str">
-        <v>13:43</v>
+        <v>13:06</v>
       </c>
       <c r="D4" t="str">
-        <v>Nap</v>
+        <v>13:45</v>
       </c>
       <c r="E4" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H4" t="str">
         <v/>
       </c>
     </row>
@@ -479,15 +518,24 @@
         <v>2026-09-01</v>
       </c>
       <c r="B5" t="str">
-        <v>14:55</v>
+        <v>14:50</v>
       </c>
       <c r="C5" t="str">
-        <v>15:38</v>
+        <v>15:06</v>
       </c>
       <c r="D5" t="str">
-        <v>Nap</v>
+        <v>15:47</v>
       </c>
       <c r="E5" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H5" t="str">
         <v/>
       </c>
     </row>
@@ -496,15 +544,24 @@
         <v>2026-09-01</v>
       </c>
       <c r="B6" t="str">
-        <v>17:08</v>
+        <v>16:57</v>
       </c>
       <c r="C6" t="str">
-        <v>17:44</v>
+        <v>17:13</v>
       </c>
       <c r="D6" t="str">
-        <v>Nap</v>
+        <v>17:57</v>
       </c>
       <c r="E6" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H6" t="str">
         <v/>
       </c>
     </row>
@@ -513,15 +570,24 @@
         <v>2026-09-01</v>
       </c>
       <c r="B7" t="str">
-        <v>19:39</v>
+        <v>19:19</v>
       </c>
       <c r="C7" t="str">
-        <v>00:55</v>
+        <v>19:37</v>
       </c>
       <c r="D7" t="str">
-        <v>Night</v>
+        <v>01:14</v>
       </c>
       <c r="E7" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
         <v>Feed</v>
       </c>
     </row>
@@ -530,15 +596,24 @@
         <v>2026-09-01</v>
       </c>
       <c r="B8" t="str">
-        <v>01:14</v>
+        <v/>
       </c>
       <c r="C8" t="str">
-        <v>06:30</v>
+        <v>01:26</v>
       </c>
       <c r="D8" t="str">
-        <v>Night</v>
+        <v>07:10</v>
       </c>
       <c r="E8" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
         <v/>
       </c>
     </row>
@@ -547,15 +622,24 @@
         <v>2026-09-02</v>
       </c>
       <c r="B9" t="str">
-        <v>08:36</v>
+        <v>08:02</v>
       </c>
       <c r="C9" t="str">
-        <v>08:58</v>
+        <v>08:20</v>
       </c>
       <c r="D9" t="str">
-        <v>Nap</v>
+        <v>08:49</v>
       </c>
       <c r="E9" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H9" t="str">
         <v/>
       </c>
     </row>
@@ -564,15 +648,24 @@
         <v>2026-09-02</v>
       </c>
       <c r="B10" t="str">
-        <v>10:51</v>
+        <v>10:37</v>
       </c>
       <c r="C10" t="str">
-        <v>11:25</v>
+        <v>10:52</v>
       </c>
       <c r="D10" t="str">
-        <v>Nap</v>
+        <v>11:38</v>
       </c>
       <c r="E10" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H10" t="str">
         <v/>
       </c>
     </row>
@@ -581,15 +674,24 @@
         <v>2026-09-02</v>
       </c>
       <c r="B11" t="str">
-        <v>13:13</v>
+        <v>12:44</v>
       </c>
       <c r="C11" t="str">
-        <v>13:57</v>
+        <v>13:00</v>
       </c>
       <c r="D11" t="str">
-        <v>Nap</v>
+        <v>13:33</v>
       </c>
       <c r="E11" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H11" t="str">
         <v/>
       </c>
     </row>
@@ -598,15 +700,24 @@
         <v>2026-09-02</v>
       </c>
       <c r="B12" t="str">
-        <v>14:49</v>
+        <v>14:35</v>
       </c>
       <c r="C12" t="str">
-        <v>15:24</v>
+        <v>14:56</v>
       </c>
       <c r="D12" t="str">
-        <v>Nap</v>
+        <v>15:26</v>
       </c>
       <c r="E12" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H12" t="str">
         <v/>
       </c>
     </row>
@@ -615,15 +726,24 @@
         <v>2026-09-02</v>
       </c>
       <c r="B13" t="str">
-        <v>17:13</v>
+        <v>16:33</v>
       </c>
       <c r="C13" t="str">
-        <v>17:54</v>
+        <v>16:50</v>
       </c>
       <c r="D13" t="str">
-        <v>Nap</v>
+        <v>17:22</v>
       </c>
       <c r="E13" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H13" t="str">
         <v/>
       </c>
     </row>
@@ -632,15 +752,24 @@
         <v>2026-09-02</v>
       </c>
       <c r="B14" t="str">
-        <v>19:37</v>
+        <v>19:03</v>
       </c>
       <c r="C14" t="str">
-        <v>01:14</v>
+        <v>19:22</v>
       </c>
       <c r="D14" t="str">
-        <v>Night</v>
+        <v>01:29</v>
       </c>
       <c r="E14" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
         <v>Feed</v>
       </c>
     </row>
@@ -649,15 +778,24 @@
         <v>2026-09-02</v>
       </c>
       <c r="B15" t="str">
-        <v>01:26</v>
+        <v/>
       </c>
       <c r="C15" t="str">
-        <v>07:10</v>
+        <v>01:47</v>
       </c>
       <c r="D15" t="str">
-        <v>Night</v>
+        <v>06:29</v>
       </c>
       <c r="E15" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
         <v/>
       </c>
     </row>
@@ -666,15 +804,24 @@
         <v>2026-09-03</v>
       </c>
       <c r="B16" t="str">
-        <v>08:40</v>
+        <v>08:15</v>
       </c>
       <c r="C16" t="str">
-        <v>09:10</v>
+        <v>08:34</v>
       </c>
       <c r="D16" t="str">
-        <v>Nap</v>
+        <v>09:09</v>
       </c>
       <c r="E16" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Fussy</v>
+      </c>
+      <c r="H16" t="str">
         <v/>
       </c>
     </row>
@@ -683,15 +830,24 @@
         <v>2026-09-03</v>
       </c>
       <c r="B17" t="str">
-        <v>10:35</v>
+        <v>10:31</v>
       </c>
       <c r="C17" t="str">
-        <v>11:04</v>
+        <v>10:51</v>
       </c>
       <c r="D17" t="str">
-        <v>Nap</v>
+        <v>11:19</v>
       </c>
       <c r="E17" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H17" t="str">
         <v/>
       </c>
     </row>
@@ -700,15 +856,24 @@
         <v>2026-09-03</v>
       </c>
       <c r="B18" t="str">
-        <v>12:58</v>
+        <v>12:34</v>
       </c>
       <c r="C18" t="str">
-        <v>13:27</v>
+        <v>12:57</v>
       </c>
       <c r="D18" t="str">
-        <v>Nap</v>
+        <v>13:41</v>
       </c>
       <c r="E18" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Fussy</v>
+      </c>
+      <c r="H18" t="str">
         <v/>
       </c>
     </row>
@@ -717,15 +882,24 @@
         <v>2026-09-03</v>
       </c>
       <c r="B19" t="str">
-        <v>15:13</v>
+        <v>14:42</v>
       </c>
       <c r="C19" t="str">
-        <v>15:50</v>
+        <v>14:57</v>
       </c>
       <c r="D19" t="str">
-        <v>Nap</v>
+        <v>15:22</v>
       </c>
       <c r="E19" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Nursing</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H19" t="str">
         <v/>
       </c>
     </row>
@@ -734,15 +908,24 @@
         <v>2026-09-03</v>
       </c>
       <c r="B20" t="str">
-        <v>17:07</v>
+        <v>16:45</v>
       </c>
       <c r="C20" t="str">
-        <v>17:53</v>
+        <v>17:04</v>
       </c>
       <c r="D20" t="str">
-        <v>Nap</v>
+        <v>17:28</v>
       </c>
       <c r="E20" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H20" t="str">
         <v/>
       </c>
     </row>
@@ -751,32 +934,50 @@
         <v>2026-09-03</v>
       </c>
       <c r="B21" t="str">
-        <v>19:08</v>
+        <v>19:28</v>
       </c>
       <c r="C21" t="str">
-        <v>00:51</v>
+        <v>19:51</v>
       </c>
       <c r="D21" t="str">
-        <v>Night</v>
+        <v>07:08</v>
       </c>
       <c r="E21" t="str">
-        <v>Feed</v>
+        <v>Night</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-09-03</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B22" t="str">
-        <v>01:00</v>
+        <v>08:25</v>
       </c>
       <c r="C22" t="str">
-        <v>06:46</v>
+        <v>08:38</v>
       </c>
       <c r="D22" t="str">
-        <v>Night</v>
+        <v>09:06</v>
       </c>
       <c r="E22" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H22" t="str">
         <v/>
       </c>
     </row>
@@ -785,15 +986,24 @@
         <v>2026-09-04</v>
       </c>
       <c r="B23" t="str">
-        <v>08:42</v>
+        <v>10:15</v>
       </c>
       <c r="C23" t="str">
-        <v>09:04</v>
+        <v>10:30</v>
       </c>
       <c r="D23" t="str">
-        <v>Nap</v>
+        <v>11:09</v>
       </c>
       <c r="E23" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H23" t="str">
         <v/>
       </c>
     </row>
@@ -802,15 +1012,24 @@
         <v>2026-09-04</v>
       </c>
       <c r="B24" t="str">
-        <v>10:41</v>
+        <v>12:44</v>
       </c>
       <c r="C24" t="str">
-        <v>11:11</v>
+        <v>13:06</v>
       </c>
       <c r="D24" t="str">
-        <v>Nap</v>
+        <v>13:33</v>
       </c>
       <c r="E24" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H24" t="str">
         <v/>
       </c>
     </row>
@@ -819,15 +1038,24 @@
         <v>2026-09-04</v>
       </c>
       <c r="B25" t="str">
-        <v>13:05</v>
+        <v>14:54</v>
       </c>
       <c r="C25" t="str">
-        <v>13:53</v>
+        <v>15:12</v>
       </c>
       <c r="D25" t="str">
-        <v>Nap</v>
+        <v>15:36</v>
       </c>
       <c r="E25" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H25" t="str">
         <v/>
       </c>
     </row>
@@ -836,15 +1064,24 @@
         <v>2026-09-04</v>
       </c>
       <c r="B26" t="str">
-        <v>15:00</v>
+        <v>16:51</v>
       </c>
       <c r="C26" t="str">
-        <v>15:25</v>
+        <v>17:13</v>
       </c>
       <c r="D26" t="str">
-        <v>Nap</v>
+        <v>17:34</v>
       </c>
       <c r="E26" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H26" t="str">
         <v/>
       </c>
     </row>
@@ -853,16 +1090,25 @@
         <v>2026-09-04</v>
       </c>
       <c r="B27" t="str">
-        <v>16:57</v>
+        <v>19:25</v>
       </c>
       <c r="C27" t="str">
-        <v>17:26</v>
+        <v>19:39</v>
       </c>
       <c r="D27" t="str">
-        <v>Nap</v>
+        <v>23:20</v>
       </c>
       <c r="E27" t="str">
-        <v/>
+        <v>Night</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v>Feed</v>
       </c>
     </row>
     <row r="28">
@@ -870,16 +1116,25 @@
         <v>2026-09-04</v>
       </c>
       <c r="B28" t="str">
-        <v>19:23</v>
+        <v/>
       </c>
       <c r="C28" t="str">
-        <v>23:20</v>
+        <v>23:39</v>
       </c>
       <c r="D28" t="str">
-        <v>Night</v>
+        <v>03:33</v>
       </c>
       <c r="E28" t="str">
-        <v>Feed</v>
+        <v>Night</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -887,32 +1142,50 @@
         <v>2026-09-04</v>
       </c>
       <c r="B29" t="str">
-        <v>23:30</v>
+        <v/>
       </c>
       <c r="C29" t="str">
-        <v>03:51</v>
+        <v>03:48</v>
       </c>
       <c r="D29" t="str">
-        <v>Night</v>
+        <v>06:28</v>
       </c>
       <c r="E29" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B30" t="str">
-        <v>04:05</v>
+        <v>08:24</v>
       </c>
       <c r="C30" t="str">
-        <v>06:47</v>
+        <v>08:46</v>
       </c>
       <c r="D30" t="str">
-        <v>Night</v>
+        <v>09:24</v>
       </c>
       <c r="E30" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H30" t="str">
         <v/>
       </c>
     </row>
@@ -921,15 +1194,24 @@
         <v>2026-09-05</v>
       </c>
       <c r="B31" t="str">
-        <v>09:11</v>
+        <v>11:50</v>
       </c>
       <c r="C31" t="str">
-        <v>10:05</v>
+        <v>12:12</v>
       </c>
       <c r="D31" t="str">
-        <v>Nap</v>
+        <v>12:48</v>
       </c>
       <c r="E31" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H31" t="str">
         <v/>
       </c>
     </row>
@@ -938,15 +1220,24 @@
         <v>2026-09-05</v>
       </c>
       <c r="B32" t="str">
-        <v>12:04</v>
+        <v>14:53</v>
       </c>
       <c r="C32" t="str">
-        <v>12:54</v>
+        <v>15:08</v>
       </c>
       <c r="D32" t="str">
-        <v>Nap</v>
+        <v>15:56</v>
       </c>
       <c r="E32" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Fussy</v>
+      </c>
+      <c r="H32" t="str">
         <v/>
       </c>
     </row>
@@ -955,15 +1246,24 @@
         <v>2026-09-05</v>
       </c>
       <c r="B33" t="str">
-        <v>15:00</v>
+        <v>16:45</v>
       </c>
       <c r="C33" t="str">
-        <v>15:56</v>
+        <v>17:07</v>
       </c>
       <c r="D33" t="str">
-        <v>Nap</v>
+        <v>17:54</v>
       </c>
       <c r="E33" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H33" t="str">
         <v/>
       </c>
     </row>
@@ -972,49 +1272,76 @@
         <v>2026-09-05</v>
       </c>
       <c r="B34" t="str">
-        <v>17:28</v>
+        <v>19:16</v>
       </c>
       <c r="C34" t="str">
-        <v>18:15</v>
+        <v>19:36</v>
       </c>
       <c r="D34" t="str">
-        <v>Nap</v>
+        <v>06:35</v>
       </c>
       <c r="E34" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B35" t="str">
-        <v>19:40</v>
+        <v>07:59</v>
       </c>
       <c r="C35" t="str">
-        <v>00:54</v>
+        <v>08:21</v>
       </c>
       <c r="D35" t="str">
-        <v>Night</v>
+        <v>08:50</v>
       </c>
       <c r="E35" t="str">
-        <v>Feed</v>
+        <v>Nap</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Nursing</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B36" t="str">
-        <v>01:07</v>
+        <v>10:42</v>
       </c>
       <c r="C36" t="str">
-        <v>06:36</v>
+        <v>10:56</v>
       </c>
       <c r="D36" t="str">
-        <v>Night</v>
+        <v>11:44</v>
       </c>
       <c r="E36" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H36" t="str">
         <v/>
       </c>
     </row>
@@ -1023,15 +1350,24 @@
         <v>2026-09-06</v>
       </c>
       <c r="B37" t="str">
-        <v>08:39</v>
+        <v>12:40</v>
       </c>
       <c r="C37" t="str">
-        <v>09:25</v>
+        <v>13:00</v>
       </c>
       <c r="D37" t="str">
-        <v>Nap</v>
+        <v>13:37</v>
       </c>
       <c r="E37" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H37" t="str">
         <v/>
       </c>
     </row>
@@ -1040,15 +1376,24 @@
         <v>2026-09-06</v>
       </c>
       <c r="B38" t="str">
-        <v>10:33</v>
+        <v>14:37</v>
       </c>
       <c r="C38" t="str">
-        <v>11:18</v>
+        <v>14:51</v>
       </c>
       <c r="D38" t="str">
-        <v>Nap</v>
+        <v>15:24</v>
       </c>
       <c r="E38" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H38" t="str">
         <v/>
       </c>
     </row>
@@ -1057,15 +1402,24 @@
         <v>2026-09-06</v>
       </c>
       <c r="B39" t="str">
-        <v>12:47</v>
+        <v>16:42</v>
       </c>
       <c r="C39" t="str">
-        <v>13:19</v>
+        <v>17:02</v>
       </c>
       <c r="D39" t="str">
-        <v>Nap</v>
+        <v>17:37</v>
       </c>
       <c r="E39" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H39" t="str">
         <v/>
       </c>
     </row>
@@ -1074,16 +1428,25 @@
         <v>2026-09-06</v>
       </c>
       <c r="B40" t="str">
-        <v>14:50</v>
+        <v>18:51</v>
       </c>
       <c r="C40" t="str">
-        <v>15:12</v>
+        <v>19:06</v>
       </c>
       <c r="D40" t="str">
-        <v>Nap</v>
+        <v>01:05</v>
       </c>
       <c r="E40" t="str">
-        <v/>
+        <v>Night</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v>Feed</v>
       </c>
     </row>
     <row r="41">
@@ -1091,49 +1454,76 @@
         <v>2026-09-06</v>
       </c>
       <c r="B41" t="str">
-        <v>17:15</v>
+        <v/>
       </c>
       <c r="C41" t="str">
-        <v>17:42</v>
+        <v>01:23</v>
       </c>
       <c r="D41" t="str">
-        <v>Nap</v>
+        <v>06:27</v>
       </c>
       <c r="E41" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B42" t="str">
-        <v>19:37</v>
+        <v>08:39</v>
       </c>
       <c r="C42" t="str">
-        <v>00:45</v>
+        <v>08:58</v>
       </c>
       <c r="D42" t="str">
-        <v>Night</v>
+        <v>09:35</v>
       </c>
       <c r="E42" t="str">
-        <v>Feed</v>
+        <v>Nap</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B43" t="str">
-        <v>01:08</v>
+        <v>11:54</v>
       </c>
       <c r="C43" t="str">
-        <v>06:51</v>
+        <v>12:05</v>
       </c>
       <c r="D43" t="str">
-        <v>Night</v>
+        <v>13:09</v>
       </c>
       <c r="E43" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H43" t="str">
         <v/>
       </c>
     </row>
@@ -1142,15 +1532,24 @@
         <v>2026-09-07</v>
       </c>
       <c r="B44" t="str">
-        <v>09:12</v>
+        <v>14:56</v>
       </c>
       <c r="C44" t="str">
-        <v>10:14</v>
+        <v>15:07</v>
       </c>
       <c r="D44" t="str">
-        <v>Nap</v>
+        <v>16:09</v>
       </c>
       <c r="E44" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H44" t="str">
         <v/>
       </c>
     </row>
@@ -1159,15 +1558,24 @@
         <v>2026-09-07</v>
       </c>
       <c r="B45" t="str">
-        <v>12:12</v>
+        <v>16:52</v>
       </c>
       <c r="C45" t="str">
-        <v>13:14</v>
+        <v>17:03</v>
       </c>
       <c r="D45" t="str">
-        <v>Nap</v>
+        <v>17:41</v>
       </c>
       <c r="E45" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Fussy</v>
+      </c>
+      <c r="H45" t="str">
         <v/>
       </c>
     </row>
@@ -1176,16 +1584,25 @@
         <v>2026-09-07</v>
       </c>
       <c r="B46" t="str">
-        <v>15:08</v>
+        <v>18:51</v>
       </c>
       <c r="C46" t="str">
-        <v>15:51</v>
+        <v>19:12</v>
       </c>
       <c r="D46" t="str">
-        <v>Nap</v>
+        <v>00:48</v>
       </c>
       <c r="E46" t="str">
-        <v/>
+        <v>Night</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G46" t="str">
+        <v/>
+      </c>
+      <c r="H46" t="str">
+        <v>Feed</v>
       </c>
     </row>
     <row r="47">
@@ -1193,49 +1610,76 @@
         <v>2026-09-07</v>
       </c>
       <c r="B47" t="str">
-        <v>17:00</v>
+        <v/>
       </c>
       <c r="C47" t="str">
-        <v>17:42</v>
+        <v>01:06</v>
       </c>
       <c r="D47" t="str">
-        <v>Nap</v>
+        <v>06:30</v>
       </c>
       <c r="E47" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-08</v>
       </c>
       <c r="B48" t="str">
-        <v>19:09</v>
+        <v>08:53</v>
       </c>
       <c r="C48" t="str">
-        <v>01:08</v>
+        <v>09:08</v>
       </c>
       <c r="D48" t="str">
-        <v>Night</v>
+        <v>09:55</v>
       </c>
       <c r="E48" t="str">
-        <v>Feed</v>
+        <v>Nap</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H48" t="str">
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-08</v>
       </c>
       <c r="B49" t="str">
-        <v>01:23</v>
+        <v>11:56</v>
       </c>
       <c r="C49" t="str">
-        <v>06:29</v>
+        <v>12:09</v>
       </c>
       <c r="D49" t="str">
-        <v>Night</v>
+        <v>13:13</v>
       </c>
       <c r="E49" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H49" t="str">
         <v/>
       </c>
     </row>
@@ -1244,15 +1688,24 @@
         <v>2026-09-08</v>
       </c>
       <c r="B50" t="str">
-        <v>09:06</v>
+        <v>14:32</v>
       </c>
       <c r="C50" t="str">
-        <v>09:48</v>
+        <v>14:49</v>
       </c>
       <c r="D50" t="str">
-        <v>Nap</v>
+        <v>15:30</v>
       </c>
       <c r="E50" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H50" t="str">
         <v/>
       </c>
     </row>
@@ -1261,15 +1714,24 @@
         <v>2026-09-08</v>
       </c>
       <c r="B51" t="str">
-        <v>12:11</v>
+        <v>16:51</v>
       </c>
       <c r="C51" t="str">
-        <v>12:53</v>
+        <v>17:08</v>
       </c>
       <c r="D51" t="str">
-        <v>Nap</v>
+        <v>18:02</v>
       </c>
       <c r="E51" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Fussy</v>
+      </c>
+      <c r="H51" t="str">
         <v/>
       </c>
     </row>
@@ -1278,16 +1740,25 @@
         <v>2026-09-08</v>
       </c>
       <c r="B52" t="str">
-        <v>14:56</v>
+        <v>19:14</v>
       </c>
       <c r="C52" t="str">
-        <v>15:58</v>
+        <v>19:26</v>
       </c>
       <c r="D52" t="str">
-        <v>Nap</v>
+        <v>22:55</v>
       </c>
       <c r="E52" t="str">
-        <v/>
+        <v>Night</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Held in arms</v>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
+      <c r="H52" t="str">
+        <v>Feed</v>
       </c>
     </row>
     <row r="53">
@@ -1295,15 +1766,24 @@
         <v>2026-09-08</v>
       </c>
       <c r="B53" t="str">
-        <v>17:04</v>
+        <v/>
       </c>
       <c r="C53" t="str">
-        <v>17:54</v>
+        <v>23:18</v>
       </c>
       <c r="D53" t="str">
-        <v>Nap</v>
+        <v>03:17</v>
       </c>
       <c r="E53" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
+      <c r="H53" t="str">
         <v/>
       </c>
     </row>
@@ -1312,15 +1792,24 @@
         <v>2026-09-08</v>
       </c>
       <c r="B54" t="str">
-        <v>19:05</v>
+        <v/>
       </c>
       <c r="C54" t="str">
-        <v>06:53</v>
+        <v>03:37</v>
       </c>
       <c r="D54" t="str">
-        <v>Night</v>
+        <v>06:15</v>
       </c>
       <c r="E54" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str">
         <v/>
       </c>
     </row>
@@ -1329,15 +1818,24 @@
         <v>2026-09-09</v>
       </c>
       <c r="B55" t="str">
-        <v>09:13</v>
+        <v>08:38</v>
       </c>
       <c r="C55" t="str">
-        <v>09:49</v>
+        <v>08:58</v>
       </c>
       <c r="D55" t="str">
-        <v>Nap</v>
+        <v>09:59</v>
       </c>
       <c r="E55" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H55" t="str">
         <v/>
       </c>
     </row>
@@ -1346,15 +1844,24 @@
         <v>2026-09-09</v>
       </c>
       <c r="B56" t="str">
-        <v>12:12</v>
+        <v>11:48</v>
       </c>
       <c r="C56" t="str">
-        <v>12:53</v>
+        <v>12:02</v>
       </c>
       <c r="D56" t="str">
-        <v>Nap</v>
+        <v>12:47</v>
       </c>
       <c r="E56" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G56" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H56" t="str">
         <v/>
       </c>
     </row>
@@ -1363,15 +1870,24 @@
         <v>2026-09-09</v>
       </c>
       <c r="B57" t="str">
-        <v>15:14</v>
+        <v>14:45</v>
       </c>
       <c r="C57" t="str">
-        <v>16:06</v>
+        <v>15:02</v>
       </c>
       <c r="D57" t="str">
-        <v>Nap</v>
+        <v>15:59</v>
       </c>
       <c r="E57" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G57" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H57" t="str">
         <v/>
       </c>
     </row>
@@ -1380,15 +1896,24 @@
         <v>2026-09-09</v>
       </c>
       <c r="B58" t="str">
-        <v>17:20</v>
+        <v>17:07</v>
       </c>
       <c r="C58" t="str">
-        <v>18:03</v>
+        <v>17:27</v>
       </c>
       <c r="D58" t="str">
-        <v>Nap</v>
+        <v>18:27</v>
       </c>
       <c r="E58" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G58" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H58" t="str">
         <v/>
       </c>
     </row>
@@ -1397,32 +1922,50 @@
         <v>2026-09-09</v>
       </c>
       <c r="B59" t="str">
-        <v>19:16</v>
+        <v>19:42</v>
       </c>
       <c r="C59" t="str">
-        <v>01:09</v>
+        <v>19:53</v>
       </c>
       <c r="D59" t="str">
-        <v>Night</v>
+        <v>06:36</v>
       </c>
       <c r="E59" t="str">
-        <v>Feed</v>
+        <v>Night</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G59" t="str">
+        <v/>
+      </c>
+      <c r="H59" t="str">
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-10</v>
       </c>
       <c r="B60" t="str">
-        <v>01:28</v>
+        <v>08:54</v>
       </c>
       <c r="C60" t="str">
-        <v>06:18</v>
+        <v>09:11</v>
       </c>
       <c r="D60" t="str">
-        <v>Night</v>
+        <v>10:07</v>
       </c>
       <c r="E60" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Nursing</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H60" t="str">
         <v/>
       </c>
     </row>
@@ -1431,15 +1974,24 @@
         <v>2026-09-10</v>
       </c>
       <c r="B61" t="str">
-        <v>09:06</v>
+        <v>11:33</v>
       </c>
       <c r="C61" t="str">
-        <v>09:56</v>
+        <v>11:51</v>
       </c>
       <c r="D61" t="str">
-        <v>Nap</v>
+        <v>12:33</v>
       </c>
       <c r="E61" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G61" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H61" t="str">
         <v/>
       </c>
     </row>
@@ -1448,15 +2000,24 @@
         <v>2026-09-10</v>
       </c>
       <c r="B62" t="str">
-        <v>11:46</v>
+        <v>14:49</v>
       </c>
       <c r="C62" t="str">
-        <v>12:24</v>
+        <v>15:04</v>
       </c>
       <c r="D62" t="str">
-        <v>Nap</v>
+        <v>16:00</v>
       </c>
       <c r="E62" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G62" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H62" t="str">
         <v/>
       </c>
     </row>
@@ -1465,15 +2026,24 @@
         <v>2026-09-10</v>
       </c>
       <c r="B63" t="str">
-        <v>15:13</v>
+        <v>17:09</v>
       </c>
       <c r="C63" t="str">
-        <v>15:52</v>
+        <v>17:26</v>
       </c>
       <c r="D63" t="str">
-        <v>Nap</v>
+        <v>18:09</v>
       </c>
       <c r="E63" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G63" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H63" t="str">
         <v/>
       </c>
     </row>
@@ -1482,32 +2052,50 @@
         <v>2026-09-10</v>
       </c>
       <c r="B64" t="str">
-        <v>17:21</v>
+        <v>18:55</v>
       </c>
       <c r="C64" t="str">
-        <v>18:23</v>
+        <v>19:14</v>
       </c>
       <c r="D64" t="str">
-        <v>Nap</v>
+        <v>06:29</v>
       </c>
       <c r="E64" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F64" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G64" t="str">
+        <v/>
+      </c>
+      <c r="H64" t="str">
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B65" t="str">
-        <v>19:07</v>
+        <v>08:52</v>
       </c>
       <c r="C65" t="str">
-        <v>07:07</v>
+        <v>09:10</v>
       </c>
       <c r="D65" t="str">
-        <v>Night</v>
+        <v>10:25</v>
       </c>
       <c r="E65" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F65" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G65" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H65" t="str">
         <v/>
       </c>
     </row>
@@ -1516,15 +2104,24 @@
         <v>2026-09-11</v>
       </c>
       <c r="B66" t="str">
-        <v>09:30</v>
+        <v>13:03</v>
       </c>
       <c r="C66" t="str">
-        <v>10:54</v>
+        <v>13:13</v>
       </c>
       <c r="D66" t="str">
-        <v>Nap</v>
+        <v>14:08</v>
       </c>
       <c r="E66" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F66" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G66" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H66" t="str">
         <v/>
       </c>
     </row>
@@ -1533,15 +2130,24 @@
         <v>2026-09-11</v>
       </c>
       <c r="B67" t="str">
-        <v>13:08</v>
+        <v>16:10</v>
       </c>
       <c r="C67" t="str">
-        <v>14:16</v>
+        <v>16:21</v>
       </c>
       <c r="D67" t="str">
-        <v>Nap</v>
+        <v>17:43</v>
       </c>
       <c r="E67" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G67" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H67" t="str">
         <v/>
       </c>
     </row>
@@ -1550,16 +2156,25 @@
         <v>2026-09-11</v>
       </c>
       <c r="B68" t="str">
-        <v>16:07</v>
+        <v>18:59</v>
       </c>
       <c r="C68" t="str">
-        <v>17:24</v>
+        <v>19:14</v>
       </c>
       <c r="D68" t="str">
-        <v>Nap</v>
+        <v>01:10</v>
       </c>
       <c r="E68" t="str">
-        <v/>
+        <v>Night</v>
+      </c>
+      <c r="F68" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G68" t="str">
+        <v/>
+      </c>
+      <c r="H68" t="str">
+        <v>Feed</v>
       </c>
     </row>
     <row r="69">
@@ -1567,49 +2182,76 @@
         <v>2026-09-11</v>
       </c>
       <c r="B69" t="str">
-        <v>19:49</v>
+        <v/>
       </c>
       <c r="C69" t="str">
-        <v>23:57</v>
+        <v>01:18</v>
       </c>
       <c r="D69" t="str">
-        <v>Night</v>
+        <v>06:16</v>
       </c>
       <c r="E69" t="str">
-        <v>Feed</v>
+        <v>Night</v>
+      </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+      <c r="G69" t="str">
+        <v/>
+      </c>
+      <c r="H69" t="str">
+        <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B70" t="str">
-        <v>00:13</v>
+        <v>08:37</v>
       </c>
       <c r="C70" t="str">
-        <v>03:37</v>
+        <v>08:55</v>
       </c>
       <c r="D70" t="str">
-        <v>Night</v>
+        <v>09:51</v>
       </c>
       <c r="E70" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G70" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H70" t="str">
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B71" t="str">
-        <v>03:54</v>
+        <v>11:53</v>
       </c>
       <c r="C71" t="str">
-        <v>06:39</v>
+        <v>12:08</v>
       </c>
       <c r="D71" t="str">
-        <v>Night</v>
+        <v>13:04</v>
       </c>
       <c r="E71" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G71" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H71" t="str">
         <v/>
       </c>
     </row>
@@ -1618,15 +2260,24 @@
         <v>2026-09-12</v>
       </c>
       <c r="B72" t="str">
-        <v>09:07</v>
+        <v>14:36</v>
       </c>
       <c r="C72" t="str">
-        <v>09:52</v>
+        <v>14:46</v>
       </c>
       <c r="D72" t="str">
-        <v>Nap</v>
+        <v>15:39</v>
       </c>
       <c r="E72" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F72" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G72" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H72" t="str">
         <v/>
       </c>
     </row>
@@ -1635,15 +2286,24 @@
         <v>2026-09-12</v>
       </c>
       <c r="B73" t="str">
-        <v>12:07</v>
+        <v>16:53</v>
       </c>
       <c r="C73" t="str">
-        <v>12:55</v>
+        <v>17:07</v>
       </c>
       <c r="D73" t="str">
-        <v>Nap</v>
+        <v>18:01</v>
       </c>
       <c r="E73" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F73" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G73" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H73" t="str">
         <v/>
       </c>
     </row>
@@ -1652,16 +2312,25 @@
         <v>2026-09-12</v>
       </c>
       <c r="B74" t="str">
-        <v>14:51</v>
+        <v>19:35</v>
       </c>
       <c r="C74" t="str">
-        <v>15:35</v>
+        <v>19:50</v>
       </c>
       <c r="D74" t="str">
-        <v>Nap</v>
+        <v>01:38</v>
       </c>
       <c r="E74" t="str">
-        <v/>
+        <v>Night</v>
+      </c>
+      <c r="F74" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G74" t="str">
+        <v/>
+      </c>
+      <c r="H74" t="str">
+        <v>Feed</v>
       </c>
     </row>
     <row r="75">
@@ -1669,32 +2338,50 @@
         <v>2026-09-12</v>
       </c>
       <c r="B75" t="str">
-        <v>17:30</v>
+        <v/>
       </c>
       <c r="C75" t="str">
-        <v>18:35</v>
+        <v>01:45</v>
       </c>
       <c r="D75" t="str">
-        <v>Nap</v>
+        <v>06:39</v>
       </c>
       <c r="E75" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F75" t="str">
+        <v/>
+      </c>
+      <c r="G75" t="str">
+        <v/>
+      </c>
+      <c r="H75" t="str">
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-09-12</v>
+        <v>2026-09-13</v>
       </c>
       <c r="B76" t="str">
-        <v>19:37</v>
+        <v>08:57</v>
       </c>
       <c r="C76" t="str">
-        <v>07:10</v>
+        <v>09:13</v>
       </c>
       <c r="D76" t="str">
-        <v>Night</v>
+        <v>10:03</v>
       </c>
       <c r="E76" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F76" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G76" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H76" t="str">
         <v/>
       </c>
     </row>
@@ -1703,15 +2390,24 @@
         <v>2026-09-13</v>
       </c>
       <c r="B77" t="str">
-        <v>08:51</v>
+        <v>11:50</v>
       </c>
       <c r="C77" t="str">
-        <v>09:45</v>
+        <v>12:07</v>
       </c>
       <c r="D77" t="str">
-        <v>Nap</v>
+        <v>13:09</v>
       </c>
       <c r="E77" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F77" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G77" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H77" t="str">
         <v/>
       </c>
     </row>
@@ -1720,15 +2416,24 @@
         <v>2026-09-13</v>
       </c>
       <c r="B78" t="str">
-        <v>11:49</v>
+        <v>14:33</v>
       </c>
       <c r="C78" t="str">
-        <v>12:39</v>
+        <v>14:50</v>
       </c>
       <c r="D78" t="str">
-        <v>Nap</v>
+        <v>15:29</v>
       </c>
       <c r="E78" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F78" t="str">
+        <v>Nursing</v>
+      </c>
+      <c r="G78" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H78" t="str">
         <v/>
       </c>
     </row>
@@ -1737,15 +2442,24 @@
         <v>2026-09-13</v>
       </c>
       <c r="B79" t="str">
-        <v>15:02</v>
+        <v>16:45</v>
       </c>
       <c r="C79" t="str">
-        <v>16:00</v>
+        <v>17:02</v>
       </c>
       <c r="D79" t="str">
-        <v>Nap</v>
+        <v>17:45</v>
       </c>
       <c r="E79" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F79" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G79" t="str">
+        <v>Fussy</v>
+      </c>
+      <c r="H79" t="str">
         <v/>
       </c>
     </row>
@@ -1754,16 +2468,25 @@
         <v>2026-09-13</v>
       </c>
       <c r="B80" t="str">
-        <v>17:28</v>
+        <v>19:04</v>
       </c>
       <c r="C80" t="str">
-        <v>18:17</v>
+        <v>19:15</v>
       </c>
       <c r="D80" t="str">
-        <v>Nap</v>
+        <v>00:33</v>
       </c>
       <c r="E80" t="str">
-        <v/>
+        <v>Night</v>
+      </c>
+      <c r="F80" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G80" t="str">
+        <v/>
+      </c>
+      <c r="H80" t="str">
+        <v>Feed</v>
       </c>
     </row>
     <row r="81">
@@ -1771,15 +2494,24 @@
         <v>2026-09-13</v>
       </c>
       <c r="B81" t="str">
-        <v>19:14</v>
+        <v/>
       </c>
       <c r="C81" t="str">
-        <v>06:25</v>
+        <v>00:43</v>
       </c>
       <c r="D81" t="str">
-        <v>Night</v>
+        <v>06:49</v>
       </c>
       <c r="E81" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F81" t="str">
+        <v/>
+      </c>
+      <c r="G81" t="str">
+        <v/>
+      </c>
+      <c r="H81" t="str">
         <v/>
       </c>
     </row>
@@ -1788,15 +2520,24 @@
         <v>2026-09-14</v>
       </c>
       <c r="B82" t="str">
-        <v>09:20</v>
+        <v>08:54</v>
       </c>
       <c r="C82" t="str">
-        <v>10:31</v>
+        <v>09:02</v>
       </c>
       <c r="D82" t="str">
-        <v>Nap</v>
+        <v>09:58</v>
       </c>
       <c r="E82" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F82" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G82" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H82" t="str">
         <v/>
       </c>
     </row>
@@ -1805,15 +2546,24 @@
         <v>2026-09-14</v>
       </c>
       <c r="B83" t="str">
-        <v>13:02</v>
+        <v>12:57</v>
       </c>
       <c r="C83" t="str">
-        <v>14:12</v>
+        <v>13:09</v>
       </c>
       <c r="D83" t="str">
-        <v>Nap</v>
+        <v>14:26</v>
       </c>
       <c r="E83" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F83" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G83" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H83" t="str">
         <v/>
       </c>
     </row>
@@ -1822,15 +2572,24 @@
         <v>2026-09-14</v>
       </c>
       <c r="B84" t="str">
-        <v>16:23</v>
+        <v>16:03</v>
       </c>
       <c r="C84" t="str">
-        <v>17:29</v>
+        <v>16:18</v>
       </c>
       <c r="D84" t="str">
-        <v>Nap</v>
+        <v>17:42</v>
       </c>
       <c r="E84" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F84" t="str">
+        <v>Nursing</v>
+      </c>
+      <c r="G84" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H84" t="str">
         <v/>
       </c>
     </row>
@@ -1839,49 +2598,76 @@
         <v>2026-09-14</v>
       </c>
       <c r="B85" t="str">
-        <v>19:43</v>
+        <v>19:27</v>
       </c>
       <c r="C85" t="str">
-        <v>23:01</v>
+        <v>19:35</v>
       </c>
       <c r="D85" t="str">
-        <v>Night</v>
+        <v>06:25</v>
       </c>
       <c r="E85" t="str">
-        <v>Feed</v>
+        <v>Night</v>
+      </c>
+      <c r="F85" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G85" t="str">
+        <v/>
+      </c>
+      <c r="H85" t="str">
+        <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-15</v>
       </c>
       <c r="B86" t="str">
-        <v>23:20</v>
+        <v>09:07</v>
       </c>
       <c r="C86" t="str">
-        <v>02:44</v>
+        <v>09:19</v>
       </c>
       <c r="D86" t="str">
-        <v>Night</v>
+        <v>10:27</v>
       </c>
       <c r="E86" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F86" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G86" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H86" t="str">
         <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2026-09-14</v>
+        <v>2026-09-15</v>
       </c>
       <c r="B87" t="str">
-        <v>02:54</v>
+        <v>12:41</v>
       </c>
       <c r="C87" t="str">
-        <v>06:48</v>
+        <v>12:49</v>
       </c>
       <c r="D87" t="str">
-        <v>Night</v>
+        <v>13:46</v>
       </c>
       <c r="E87" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F87" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G87" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H87" t="str">
         <v/>
       </c>
     </row>
@@ -1890,15 +2676,24 @@
         <v>2026-09-15</v>
       </c>
       <c r="B88" t="str">
-        <v>09:20</v>
+        <v>15:58</v>
       </c>
       <c r="C88" t="str">
-        <v>10:28</v>
+        <v>16:06</v>
       </c>
       <c r="D88" t="str">
-        <v>Nap</v>
+        <v>17:20</v>
       </c>
       <c r="E88" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F88" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G88" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H88" t="str">
         <v/>
       </c>
     </row>
@@ -1907,49 +2702,76 @@
         <v>2026-09-15</v>
       </c>
       <c r="B89" t="str">
-        <v>12:47</v>
+        <v>19:32</v>
       </c>
       <c r="C89" t="str">
-        <v>14:05</v>
+        <v>19:47</v>
       </c>
       <c r="D89" t="str">
-        <v>Nap</v>
+        <v>06:18</v>
       </c>
       <c r="E89" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F89" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G89" t="str">
+        <v/>
+      </c>
+      <c r="H89" t="str">
         <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B90" t="str">
-        <v>16:25</v>
+        <v>08:58</v>
       </c>
       <c r="C90" t="str">
-        <v>17:47</v>
+        <v>09:12</v>
       </c>
       <c r="D90" t="str">
-        <v>Nap</v>
+        <v>10:34</v>
       </c>
       <c r="E90" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F90" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G90" t="str">
+        <v>Fussy</v>
+      </c>
+      <c r="H90" t="str">
         <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B91" t="str">
-        <v>19:51</v>
+        <v>12:58</v>
       </c>
       <c r="C91" t="str">
-        <v>07:13</v>
+        <v>13:04</v>
       </c>
       <c r="D91" t="str">
-        <v>Night</v>
+        <v>14:12</v>
       </c>
       <c r="E91" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F91" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G91" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H91" t="str">
         <v/>
       </c>
     </row>
@@ -1958,15 +2780,24 @@
         <v>2026-09-16</v>
       </c>
       <c r="B92" t="str">
-        <v>09:01</v>
+        <v>16:08</v>
       </c>
       <c r="C92" t="str">
-        <v>10:19</v>
+        <v>16:23</v>
       </c>
       <c r="D92" t="str">
-        <v>Nap</v>
+        <v>17:25</v>
       </c>
       <c r="E92" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F92" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G92" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H92" t="str">
         <v/>
       </c>
     </row>
@@ -1975,16 +2806,25 @@
         <v>2026-09-16</v>
       </c>
       <c r="B93" t="str">
-        <v>13:03</v>
+        <v>19:15</v>
       </c>
       <c r="C93" t="str">
-        <v>14:20</v>
+        <v>19:28</v>
       </c>
       <c r="D93" t="str">
-        <v>Nap</v>
+        <v>23:51</v>
       </c>
       <c r="E93" t="str">
-        <v/>
+        <v>Night</v>
+      </c>
+      <c r="F93" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G93" t="str">
+        <v/>
+      </c>
+      <c r="H93" t="str">
+        <v>Feed</v>
       </c>
     </row>
     <row r="94">
@@ -1992,15 +2832,24 @@
         <v>2026-09-16</v>
       </c>
       <c r="B94" t="str">
-        <v>16:27</v>
+        <v/>
       </c>
       <c r="C94" t="str">
-        <v>17:23</v>
+        <v>00:13</v>
       </c>
       <c r="D94" t="str">
-        <v>Nap</v>
+        <v>04:33</v>
       </c>
       <c r="E94" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F94" t="str">
+        <v/>
+      </c>
+      <c r="G94" t="str">
+        <v/>
+      </c>
+      <c r="H94" t="str">
         <v/>
       </c>
     </row>
@@ -2009,49 +2858,76 @@
         <v>2026-09-16</v>
       </c>
       <c r="B95" t="str">
-        <v>19:12</v>
+        <v/>
       </c>
       <c r="C95" t="str">
-        <v>22:16</v>
+        <v>04:54</v>
       </c>
       <c r="D95" t="str">
-        <v>Night</v>
+        <v>07:08</v>
       </c>
       <c r="E95" t="str">
-        <v>Feed</v>
+        <v>Night</v>
+      </c>
+      <c r="F95" t="str">
+        <v/>
+      </c>
+      <c r="G95" t="str">
+        <v/>
+      </c>
+      <c r="H95" t="str">
+        <v/>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B96" t="str">
-        <v>22:33</v>
+        <v>09:11</v>
       </c>
       <c r="C96" t="str">
-        <v>02:51</v>
+        <v>09:23</v>
       </c>
       <c r="D96" t="str">
-        <v>Night</v>
+        <v>10:47</v>
       </c>
       <c r="E96" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F96" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G96" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H96" t="str">
         <v/>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B97" t="str">
-        <v>03:00</v>
+        <v>12:48</v>
       </c>
       <c r="C97" t="str">
-        <v>06:20</v>
+        <v>12:55</v>
       </c>
       <c r="D97" t="str">
-        <v>Night</v>
+        <v>14:16</v>
       </c>
       <c r="E97" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F97" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G97" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H97" t="str">
         <v/>
       </c>
     </row>
@@ -2060,15 +2936,24 @@
         <v>2026-09-17</v>
       </c>
       <c r="B98" t="str">
-        <v>09:04</v>
+        <v>16:11</v>
       </c>
       <c r="C98" t="str">
-        <v>10:05</v>
+        <v>16:24</v>
       </c>
       <c r="D98" t="str">
-        <v>Nap</v>
+        <v>17:33</v>
       </c>
       <c r="E98" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F98" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G98" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H98" t="str">
         <v/>
       </c>
     </row>
@@ -2077,16 +2962,25 @@
         <v>2026-09-17</v>
       </c>
       <c r="B99" t="str">
-        <v>13:05</v>
+        <v>19:06</v>
       </c>
       <c r="C99" t="str">
-        <v>14:07</v>
+        <v>19:17</v>
       </c>
       <c r="D99" t="str">
-        <v>Nap</v>
+        <v>23:33</v>
       </c>
       <c r="E99" t="str">
-        <v/>
+        <v>Night</v>
+      </c>
+      <c r="F99" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G99" t="str">
+        <v/>
+      </c>
+      <c r="H99" t="str">
+        <v>Feed</v>
       </c>
     </row>
     <row r="100">
@@ -2094,15 +2988,24 @@
         <v>2026-09-17</v>
       </c>
       <c r="B100" t="str">
-        <v>16:14</v>
+        <v/>
       </c>
       <c r="C100" t="str">
-        <v>17:39</v>
+        <v>23:55</v>
       </c>
       <c r="D100" t="str">
-        <v>Nap</v>
+        <v>04:11</v>
       </c>
       <c r="E100" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F100" t="str">
+        <v/>
+      </c>
+      <c r="G100" t="str">
+        <v/>
+      </c>
+      <c r="H100" t="str">
         <v/>
       </c>
     </row>
@@ -2111,15 +3014,24 @@
         <v>2026-09-17</v>
       </c>
       <c r="B101" t="str">
-        <v>19:26</v>
+        <v/>
       </c>
       <c r="C101" t="str">
-        <v>07:01</v>
+        <v>04:20</v>
       </c>
       <c r="D101" t="str">
-        <v>Night</v>
+        <v>06:50</v>
       </c>
       <c r="E101" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F101" t="str">
+        <v/>
+      </c>
+      <c r="G101" t="str">
+        <v/>
+      </c>
+      <c r="H101" t="str">
         <v/>
       </c>
     </row>
@@ -2128,15 +3040,24 @@
         <v>2026-09-18</v>
       </c>
       <c r="B102" t="str">
-        <v>09:12</v>
+        <v>09:08</v>
       </c>
       <c r="C102" t="str">
-        <v>10:19</v>
+        <v>09:17</v>
       </c>
       <c r="D102" t="str">
-        <v>Nap</v>
+        <v>10:26</v>
       </c>
       <c r="E102" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F102" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G102" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H102" t="str">
         <v/>
       </c>
     </row>
@@ -2145,15 +3066,24 @@
         <v>2026-09-18</v>
       </c>
       <c r="B103" t="str">
-        <v>12:47</v>
+        <v>12:51</v>
       </c>
       <c r="C103" t="str">
-        <v>13:49</v>
+        <v>13:01</v>
       </c>
       <c r="D103" t="str">
-        <v>Nap</v>
+        <v>14:08</v>
       </c>
       <c r="E103" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F103" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G103" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H103" t="str">
         <v/>
       </c>
     </row>
@@ -2162,15 +3092,24 @@
         <v>2026-09-18</v>
       </c>
       <c r="B104" t="str">
-        <v>16:24</v>
+        <v>16:15</v>
       </c>
       <c r="C104" t="str">
-        <v>17:48</v>
+        <v>16:23</v>
       </c>
       <c r="D104" t="str">
-        <v>Nap</v>
+        <v>17:27</v>
       </c>
       <c r="E104" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F104" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G104" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H104" t="str">
         <v/>
       </c>
     </row>
@@ -2179,15 +3118,24 @@
         <v>2026-09-18</v>
       </c>
       <c r="B105" t="str">
-        <v>19:13</v>
+        <v>19:41</v>
       </c>
       <c r="C105" t="str">
-        <v>06:46</v>
+        <v>19:52</v>
       </c>
       <c r="D105" t="str">
-        <v>Night</v>
+        <v>06:34</v>
       </c>
       <c r="E105" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F105" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G105" t="str">
+        <v/>
+      </c>
+      <c r="H105" t="str">
         <v/>
       </c>
     </row>
@@ -2196,15 +3144,24 @@
         <v>2026-09-19</v>
       </c>
       <c r="B106" t="str">
-        <v>09:04</v>
+        <v>09:13</v>
       </c>
       <c r="C106" t="str">
-        <v>10:05</v>
+        <v>09:19</v>
       </c>
       <c r="D106" t="str">
-        <v>Nap</v>
+        <v>10:31</v>
       </c>
       <c r="E106" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F106" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G106" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H106" t="str">
         <v/>
       </c>
     </row>
@@ -2213,15 +3170,24 @@
         <v>2026-09-19</v>
       </c>
       <c r="B107" t="str">
-        <v>13:03</v>
+        <v>12:42</v>
       </c>
       <c r="C107" t="str">
-        <v>14:03</v>
+        <v>12:55</v>
       </c>
       <c r="D107" t="str">
-        <v>Nap</v>
+        <v>14:09</v>
       </c>
       <c r="E107" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F107" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G107" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H107" t="str">
         <v/>
       </c>
     </row>
@@ -2230,15 +3196,24 @@
         <v>2026-09-19</v>
       </c>
       <c r="B108" t="str">
-        <v>16:02</v>
+        <v>16:05</v>
       </c>
       <c r="C108" t="str">
-        <v>17:05</v>
+        <v>16:10</v>
       </c>
       <c r="D108" t="str">
-        <v>Nap</v>
+        <v>17:17</v>
       </c>
       <c r="E108" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F108" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G108" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H108" t="str">
         <v/>
       </c>
     </row>
@@ -2247,15 +3222,24 @@
         <v>2026-09-19</v>
       </c>
       <c r="B109" t="str">
-        <v>19:37</v>
+        <v>19:19</v>
       </c>
       <c r="C109" t="str">
-        <v>06:44</v>
+        <v>19:29</v>
       </c>
       <c r="D109" t="str">
-        <v>Night</v>
+        <v>06:20</v>
       </c>
       <c r="E109" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F109" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G109" t="str">
+        <v/>
+      </c>
+      <c r="H109" t="str">
         <v/>
       </c>
     </row>
@@ -2264,15 +3248,24 @@
         <v>2026-09-20</v>
       </c>
       <c r="B110" t="str">
-        <v>09:30</v>
+        <v>09:02</v>
       </c>
       <c r="C110" t="str">
-        <v>10:27</v>
+        <v>09:14</v>
       </c>
       <c r="D110" t="str">
-        <v>Nap</v>
+        <v>10:12</v>
       </c>
       <c r="E110" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F110" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G110" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H110" t="str">
         <v/>
       </c>
     </row>
@@ -2281,15 +3274,24 @@
         <v>2026-09-20</v>
       </c>
       <c r="B111" t="str">
-        <v>12:57</v>
+        <v>12:41</v>
       </c>
       <c r="C111" t="str">
-        <v>14:01</v>
+        <v>12:49</v>
       </c>
       <c r="D111" t="str">
-        <v>Nap</v>
+        <v>13:50</v>
       </c>
       <c r="E111" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F111" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G111" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H111" t="str">
         <v/>
       </c>
     </row>
@@ -2298,15 +3300,24 @@
         <v>2026-09-20</v>
       </c>
       <c r="B112" t="str">
-        <v>16:00</v>
+        <v>16:05</v>
       </c>
       <c r="C112" t="str">
-        <v>16:55</v>
+        <v>16:17</v>
       </c>
       <c r="D112" t="str">
-        <v>Nap</v>
+        <v>17:35</v>
       </c>
       <c r="E112" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F112" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G112" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H112" t="str">
         <v/>
       </c>
     </row>
@@ -2315,49 +3326,76 @@
         <v>2026-09-20</v>
       </c>
       <c r="B113" t="str">
-        <v>19:26</v>
+        <v>18:58</v>
       </c>
       <c r="C113" t="str">
-        <v>23:43</v>
+        <v>19:11</v>
       </c>
       <c r="D113" t="str">
-        <v>Night</v>
+        <v>06:59</v>
       </c>
       <c r="E113" t="str">
-        <v>Feed</v>
+        <v>Night</v>
+      </c>
+      <c r="F113" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G113" t="str">
+        <v/>
+      </c>
+      <c r="H113" t="str">
+        <v/>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="B114" t="str">
-        <v>00:03</v>
+        <v>09:16</v>
       </c>
       <c r="C114" t="str">
-        <v>03:52</v>
+        <v>09:29</v>
       </c>
       <c r="D114" t="str">
-        <v>Night</v>
+        <v>10:33</v>
       </c>
       <c r="E114" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F114" t="str">
+        <v>Patting</v>
+      </c>
+      <c r="G114" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H114" t="str">
         <v/>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="B115" t="str">
-        <v>04:14</v>
+        <v>12:42</v>
       </c>
       <c r="C115" t="str">
-        <v>07:10</v>
+        <v>12:54</v>
       </c>
       <c r="D115" t="str">
-        <v>Night</v>
+        <v>14:15</v>
       </c>
       <c r="E115" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F115" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G115" t="str">
+        <v>Good</v>
+      </c>
+      <c r="H115" t="str">
         <v/>
       </c>
     </row>
@@ -2366,15 +3404,24 @@
         <v>2026-09-21</v>
       </c>
       <c r="B116" t="str">
-        <v>09:29</v>
+        <v>15:56</v>
       </c>
       <c r="C116" t="str">
-        <v>10:48</v>
+        <v>16:07</v>
       </c>
       <c r="D116" t="str">
-        <v>Nap</v>
+        <v>17:18</v>
       </c>
       <c r="E116" t="str">
+        <v>Nap</v>
+      </c>
+      <c r="F116" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G116" t="str">
+        <v>Crying</v>
+      </c>
+      <c r="H116" t="str">
         <v/>
       </c>
     </row>
@@ -2383,55 +3430,30 @@
         <v>2026-09-21</v>
       </c>
       <c r="B117" t="str">
-        <v>13:05</v>
+        <v>19:31</v>
       </c>
       <c r="C117" t="str">
-        <v>14:17</v>
+        <v>19:34</v>
       </c>
       <c r="D117" t="str">
-        <v>Nap</v>
+        <v>06:33</v>
       </c>
       <c r="E117" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="str">
-        <v>2026-09-21</v>
-      </c>
-      <c r="B118" t="str">
-        <v>16:10</v>
-      </c>
-      <c r="C118" t="str">
-        <v>17:17</v>
-      </c>
-      <c r="D118" t="str">
-        <v>Nap</v>
-      </c>
-      <c r="E118" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="str">
-        <v>2026-09-21</v>
-      </c>
-      <c r="B119" t="str">
-        <v>19:30</v>
-      </c>
-      <c r="C119" t="str">
-        <v>06:49</v>
-      </c>
-      <c r="D119" t="str">
-        <v>Night</v>
-      </c>
-      <c r="E119" t="str">
+        <v>Night</v>
+      </c>
+      <c r="F117" t="str">
+        <v>Independently</v>
+      </c>
+      <c r="G117" t="str">
+        <v/>
+      </c>
+      <c r="H117" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E119"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H117"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>